<commit_message>
derse hoca ve sınıf atama suan cok guzel calısıyor
</commit_message>
<xml_diff>
--- a/app/edusync_import.xlsx
+++ b/app/edusync_import.xlsx
@@ -510,153 +510,153 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>CNG 104</t>
+          <t>CNG 101</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Programming</t>
+          <t>Introduction to Computer Engineering</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Assist. Prof. Porkodi Sivaram</t>
+          <t>Assist. Prof. Celal Alagoz</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>EEE 102</t>
+          <t>CNG 104</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Circuit Theory I</t>
+          <t>Programming</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Assist. Prof. Recep Emir</t>
+          <t>Assist. Prof. Porkodi Sivaram</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>EEE 204</t>
+          <t>EEE 102</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Digital System Design</t>
+          <t>Circuit Theory I</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Assist. Prof. Nurbanu Guzey</t>
+          <t>Assist. Prof. Recep Emir</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>EEE 206</t>
+          <t>EEE 204</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Microprocessors</t>
+          <t>Digital System Design</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Assist. Prof. Celal Alagoz</t>
+          <t>Assist. Prof. Nurbanu Guzey</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>CNG 244</t>
+          <t>EEE 206</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Operating Systems</t>
+          <t>Microprocessors</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Prof. Sivaram Murugan</t>
+          <t>Assist. Prof. Celal Alagoz</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>CNG 212</t>
+          <t>CNG 244</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Programming Languages</t>
+          <t>Operating Systems</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Assoc. Prof. Farhan Aadil</t>
+          <t>Prof. Sivaram Murugan</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>CNG 342</t>
+          <t>CNG 212</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Data Communication and Computer Networks</t>
+          <t>Programming Languages</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Assist. Prof. Rezan Bakir</t>
+          <t>Assoc. Prof. Farhan Aadil</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>CNG 346</t>
+          <t>CNG 342</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Mobile Programming</t>
+          <t>Computer Networks</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Assoc. Prof. Farhan Aadil</t>
+          <t>Assist. Prof. Rezan Bakir</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>CNG 344</t>
+          <t>CNG 346</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Information Security</t>
+          <t>Mobile Programming</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Assist. Prof. Porkodi Sivaram</t>
+          <t>Assoc. Prof. Farhan Aadil</t>
         </is>
       </c>
     </row>
@@ -685,7 +685,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Artificial Intelligence Agents and Applications</t>
+          <t>AI Agents and Applications</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -702,7 +702,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Computer Networks</t>
+          <t>Computer Networks II</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">

</xml_diff>